<commit_message>
fix: update Reading3 Q1-Q8 prompts with contextual gap format
Agent-Logs-Url: https://github.com/academiaohara/cambridge-exams/sessions/a7ac9a64-ee42-428d-88a2-e3d2ff8005e6

Co-authored-by: academiaohara <253255719+academiaohara@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/social media/B2/Reading3.xlsx
+++ b/social media/B2/Reading3.xlsx
@@ -587,42 +587,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TREAT</t>
+          <t>fashionable. These (17) (TREAT) involve a person placing their feet in a tank of water full of tiny Garra rufa fish. The fish nibble the person’s feet, eating and removing the dead skin. The benefits are said to be</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>treatments involve a person placing their feet in a tank of water full of tiny Garra rufa fish. The fish nibble the person’s feet, eating and removing the dead skin. The benefits are said to be (18) (NUMBER); the pedicures seem to stimulate blood flow and improve</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CIRCULATE</t>
+          <t>numerous; the pedicures seem to stimulate blood flow and improve (19) (CIRCULATE), they make the skin feel soft and clean, and they can help eliminate foot odour. Indeed, the</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>POPULAR</t>
+          <t>circulation, they make the skin feel soft and clean, and they can help eliminate foot odour. Indeed, the (20) (POPULAR) of fish pedicures has exploded in the past few years and dozens of centres have opened nationwide. However, there have been reports claiming that there is a</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>POSSIBLE</t>
+          <t>popularity of fish pedicures has exploded in the past few years and dozens of centres have opened nationwide. However, there have been reports claiming that there is a (21) (POSSIBLE) that people could pick up an</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>INFECT</t>
+          <t>possibility that people could pick up an (22) (INFECT) from the water, the fish or other patients’ feet. Other experts claim the risk is small and that reports like these</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ESTIMATE</t>
+          <t>infection from the water, the fish or other patients’ feet. Other experts claim the risk is small and that reports like these (23) (ESTIMATE) the problem. However, they do recommend that centres undergo regular inspections to make sure the pedicures are not being carried out in</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>HYGIENE</t>
+          <t>overestimate the problem. However, they do recommend that centres undergo regular inspections to make sure the pedicures are not being carried out in (24) (HYGIENE) conditions.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -712,42 +712,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>generally agree that regular physical activity is one of the most effective ways to improve health. Many adults, however, are completely (17) (ACTIVE) and spend most of their day sitting down. Even moderate exercise can lead to clear</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IMPROVE</t>
+          <t>inactive and spend most of their day sitting down. Even moderate exercise can lead to clear (18) (IMPROVE) in both energy levels and mood. People who work out regularly tend to develop greater physical</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>STRONG</t>
+          <t>improvement in both energy levels and mood. People who work out regularly tend to develop greater physical (19) (STRONG) and are less likely to fall ill. Activities such as walking or swimming are highly</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BENEFIT</t>
+          <t>strength and are less likely to fall ill. Activities such as walking or swimming are highly (20) (BENEFIT) because they require little or no equipment. The main</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>DIFFICULT</t>
+          <t>beneficial because they require little or no equipment. The main (21) (DIFFICULT) for most people is finding the motivation to start and stick to a routine. Some people feel</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>COMFORT</t>
+          <t>difficulty for most people is finding the motivation to start and stick to a routine. Some people feel (22) (COMFORT) exercising in public, which is why home workouts have grown in popularity. Health experts</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>uncomfortable exercising in public, which is why home workouts have grown in popularity. Health experts (23) (REGULAR) advise at least 150 minutes of moderate activity per week. Those who ignore this advice risk leading an</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>HEALTH</t>
+          <t>regularly advise at least 150 minutes of moderate activity per week. Those who ignore this advice risk leading an (24) (HEALTH) lifestyle with serious long-term consequences.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -837,42 +837,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CONNECT</t>
+          <t>widely changed how people communicate and share information. Every day, millions of posts are shared across platforms, creating a powerful (17) (CONNECT) between users from different countries. Unfortunately,</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>connection between users from different countries. Unfortunately, (18) (RELY) content can spread rapidly, as many users share posts without checking facts. In spite of this, genuine</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FRIEND</t>
+          <t>unreliable content can spread rapidly, as many users share posts without checking facts. In spite of this, genuine (19) (FRIEND) can form through online communities built around shared interests. For businesses, social media offers an</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>EXPENSE</t>
+          <t>friendship can form through online communities built around shared interests. For businesses, social media offers an (20) (EXPENSE) way to reach large audiences worldwide. Young users must behave</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>inexpensive way to reach large audiences worldwide. Young users must behave (21) (RESPONSIBLE) online, as careless comments can have lasting negative effects. Research shows that heavy use of social media is linked to increased feelings of</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>DEPRESS</t>
+          <t>responsibly online, as careless comments can have lasting negative effects. Research shows that heavy use of social media is linked to increased feelings of (22) (DEPRESS) and</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>LONELY</t>
+          <t>depression and (23) (LONELY), particularly among teenagers. Experts therefore encourage greater</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>loneliness, particularly among teenagers. Experts therefore encourage greater (24) (AWARE) of these risks and recommend limiting daily screen time to protect mental wellbeing.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -962,42 +962,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DISCOVER</t>
+          <t>scientific endeavours of the modern age. Since the first satellites were launched in the 1950s, humans have made extraordinary (17) (DISCOVER) about our solar system and beyond. The journey to other planets is</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>discoveries about our solar system and beyond. The journey to other planets is (18) (FASCINATE) to scientists and the general public alike. Recent advances in</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>TECHNOLOGY</t>
+          <t>fascinating to scientists and the general public alike. Recent advances in (19) (TECHNOLOGY) equipment have made space missions cheaper and more reliable. Many people once thought it was</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>POSSIBLE</t>
+          <t>technological equipment have made space missions cheaper and more reliable. Many people once thought it was (20) (POSSIBLE) to land on the moon, yet the event proved them wrong. The</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ACHIEVE</t>
+          <t>impossible to land on the moon, yet the event proved them wrong. The (21) (ACHIEVE) of sending humans into space required enormous courage and innovation. Plans for</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>EXPLORE</t>
+          <t>achievement of sending humans into space required enormous courage and innovation. Plans for (22) (EXPLORE) of Mars are already being developed by several international agencies. The photographs sent back from space probes are deeply</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>IMPRESS</t>
+          <t>exploration of Mars are already being developed by several international agencies. The photographs sent back from space probes are deeply (23) (IMPRESS). However, space programmes remain highly</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>EXPENSE</t>
+          <t>impressive. However, space programmes remain highly (24) (EXPENSE), raising questions about whether the funding could be better spent on Earth.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1087,42 +1087,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>POLLUTE</t>
+          <t>environmental damage caused by human activity is now one of the most serious issues facing the planet. Air and water (17) (POLLUTE) affects millions of people and countless species worldwide. The burning of fossil fuels releases gases that are deeply</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HARM</t>
+          <t>pollution affects millions of people and countless species worldwide. The burning of fossil fuels releases gases that are deeply (18) (HARM) to the atmosphere, contributing to climate change. Many animal and plant species are now</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>THREAT</t>
+          <t>harmful to the atmosphere, contributing to climate change. Many animal and plant species are now (19) (THREAT) as their natural habitats are destroyed. Forests and oceans play a vital role in maintaining</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>NATURE</t>
+          <t>threatened as their natural habitats are destroyed. Forests and oceans play a vital role in maintaining (20) (NATURE) balance and biodiversity. Moving towards</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>natural balance and biodiversity. Moving towards (21) (SUSTAIN) sources of energy is essential to reduce our carbon footprint.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CARE</t>
+          <t>sustainable sources of energy is essential to reduce our carbon footprint. (22) (CARE) disposal of waste products continues to damage both land and sea. Greater</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PROTECT</t>
+          <t>careless disposal of waste products continues to damage both land and sea. Greater (23) (PROTECT) of national parks and marine areas is needed urgently. The</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>INDUSTRY</t>
+          <t>protection of national parks and marine areas is needed urgently. The (24) (INDUSTRY) sector must adopt greener practices if future generations are to enjoy a healthy planet.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1212,42 +1212,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TRADITION</t>
+          <t>education has transformed how people gain knowledge and qualifications. In the past, classroom teaching was the only option, but today there are many (17) (TRADITION) and digital alternatives available to learners. Online courses are highly</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ACCESS</t>
+          <t>traditional and digital alternatives available to learners. Online courses are highly (18) (ACCESS) to anyone with an internet connection, removing geographical barriers. However, one major</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ADVANTAGE</t>
+          <t>accessible to anyone with an internet connection, removing geographical barriers. However, one major (19) (ADVANTAGE) is that students may feel isolated without face-to-face contact with peers. Studying from home requires great</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>FLEXIBLE</t>
+          <t>disadvantage is that students may feel isolated without face-to-face contact with peers. Studying from home requires great (20) (FLEXIBLE), as learners must organise their own schedules. Without strong</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>MOTIVATE</t>
+          <t>flexibility, as learners must organise their own schedules. Without strong (21) (MOTIVATE), many students struggle to complete online programmes successfully. The lack of direct</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>INTERACT</t>
+          <t>motivation, many students struggle to complete online programmes successfully. The lack of direct (22) (INTERACT) with teachers can make it harder to ask questions and get immediate support. An</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>ABLE</t>
+          <t>interaction with teachers can make it harder to ask questions and get immediate support. An (23) (ABLE) to stay focused is another common challenge reported by online learners. Despite these issues, many students find that their</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ACHIEVE</t>
+          <t>inability to stay focused is another common challenge reported by online learners. Despite these issues, many students find that their (24) (ACHIEVE) through digital learning are just as impressive as those gained in traditional classrooms.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1337,42 +1337,42 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BENEFIT</t>
+          <t>voluntary basis, helping others without expecting payment. The (17) (BENEFIT) effects of volunteering are well documented and include improved mental health and greater social connection. Volunteers often work within local communities, assisting with activities that may otherwise go unfunded. Running a successful volunteer programme requires careful</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ORGANISE</t>
+          <t>beneficial effects of volunteering are well documented and include improved mental health and greater social connection. Volunteers often work within local communities, assisting with activities that may otherwise go unfunded. Running a successful volunteer programme requires careful (18) (ORGANISE) and strong leadership skills. Most volunteers report a deep sense of personal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>organisation and strong leadership skills. Most volunteers report a deep sense of personal (19) (SATISFY) from knowing that their efforts have made a positive difference. The skills gained through volunteering are</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>satisfaction from knowing that their efforts have made a positive difference. The skills gained through volunteering are (20) (VALUE) and are increasingly recognised by employers. Some volunteers are</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>EMPLOY</t>
+          <t>valuable and are increasingly recognised by employers. Some volunteers are (21) (EMPLOY) and use their experience to develop new abilities and improve career prospects. Charities rely on</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>SUPPORT</t>
+          <t>unemployed and use their experience to develop new abilities and improve career prospects. Charities rely on (22) (SUPPORT) networks of volunteers to deliver services that would otherwise be unaffordable. Taking on a volunteer role requires personal</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>supportive networks of volunteers to deliver services that would otherwise be unaffordable. Taking on a volunteer role requires personal (23) (RESPONSIBLE) and a genuine</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>COMMIT</t>
+          <t>responsibility and a genuine (24) (COMMIT) to the cause.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1462,42 +1462,42 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>POLLUTE</t>
+          <t>significant environmental challenges of our time. The (17) (POLLUTE) of oceans and rivers by plastic has reached alarming levels in recent decades. Global</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PRODUCE</t>
+          <t>pollution of oceans and rivers by plastic has reached alarming levels in recent decades. Global (18) (PRODUCE) of single-use plastics continues to rise despite international warnings. The chemicals released by plastic waste are deeply</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HARM</t>
+          <t>production of single-use plastics continues to rise despite international warnings. The chemicals released by plastic waste are deeply (19) (HARM) to marine life and can enter the food chain. The current model of consuming and discarding plastic is clearly</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>harmful to marine life and can enter the food chain. The current model of consuming and discarding plastic is clearly (20) (SUSTAIN) and must change urgently. Scientists and governments are working together to find a lasting</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SOLVE</t>
+          <t>unsustainable and must change urgently. Scientists and governments are working together to find a lasting (21) (SOLVE) to the crisis. Much of the problem stems from</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>solution to the crisis. Much of the problem stems from (22) (RESPONSIBLE) disposal of waste by both individuals and businesses. Greater public</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>irresponsible disposal of waste by both individuals and businesses. Greater public (23) (AWARE) of the issue is essential, as many people do not realise how serious the situation has become. Better</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>MANAGE</t>
+          <t>awareness of the issue is essential, as many people do not realise how serious the situation has become. Better (24) (MANAGE) of plastic waste through improved recycling systems is now considered a global priority.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1587,42 +1587,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ACCURATE</t>
+          <t>revolutionary changes to many aspects of modern life. AI systems now perform complex tasks with remarkable (17) (ACCURATE), sometimes matching or exceeding human performance. One</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CONSIDER</t>
+          <t>accuracy, sometimes matching or exceeding human performance. One (18) (CONSIDER) concern is how AI might affect levels of human</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CREATE</t>
+          <t>considerable concern is how AI might affect levels of human (19) (CREATE) in fields such as art and music. The rise of</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AUTOMATE</t>
+          <t>creativity in fields such as art and music. The rise of (20) (AUTOMATE) in manufacturing means fewer workers are needed on production lines, raising worries about future</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>EMPLOY</t>
+          <t>automation in manufacturing means fewer workers are needed on production lines, raising worries about future (21) (EMPLOY). Developers must ensure AI operates within</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ETHICS</t>
+          <t>employment. Developers must ensure AI operates within (22) (ETHICS) boundaries and respects individual rights. The</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>ethical boundaries and respects individual rights. The (23) (SECURE) of personal data collected by AI platforms must also be carefully managed to prevent misuse. Some scientists warn that machines with</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>HUMAN</t>
+          <t>security of personal data collected by AI platforms must also be carefully managed to prevent misuse. Some scientists warn that machines with (24) (HUMAN) levels of intelligence, operating beyond human control, could pose a serious threat to society.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1712,42 +1712,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ESSENCE</t>
+          <t>scientific curiosity – it is a biological necessity. Modern research confirms that getting enough rest is truly (17) (ESSENCE) for both physical and mental wellbeing. Without adequate sleep, people suffer from extreme</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TIRE</t>
+          <t>essential for both physical and mental wellbeing. Without adequate sleep, people suffer from extreme (18) (TIRE) that can make even simple tasks difficult. Poor sleep also reduces the</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CONCENTRATE</t>
+          <t>tiredness that can make even simple tasks difficult. Poor sleep also reduces the (19) (CONCENTRATE) needed to study or work effectively. Regular, restful sleep helps maintain a</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HEALTH</t>
+          <t>concentration needed to study or work effectively. Regular, restful sleep helps maintain a (20) (HEALTH) immune system and reduces the risk of many serious diseases. The body follows an internal</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>REGULATE</t>
+          <t>healthy immune system and reduces the risk of many serious diseases. The body follows an internal (21) (REGULATE) system known as the circadian rhythm, which controls when we feel sleepy or alert.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CONSEQUENCE</t>
+          <t>regulation system known as the circadian rhythm, which controls when we feel sleepy or alert. (22) (CONSEQUENCE), when this rhythm is disrupted by late nights or travel, people often feel confused and unwell. Research has shown that even one</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SUFFICIENT</t>
+          <t>consequently, when this rhythm is disrupted by late nights or travel, people often feel confused and unwell. Research has shown that even one (23) (SUFFICIENT) night of sleep can affect memory, judgement, and reaction time. Long-term sleep deprivation can lead to serious medical conditions and</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>FUNCTION</t>
+          <t>insufficient night of sleep can affect memory, judgement, and reaction time. Long-term sleep deprivation can lead to serious medical conditions and (24) (FUNCTION) of normal mental processes.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1837,42 +1837,42 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PRESERVE</t>
+          <t>historical resources that societies possess. The (17) (PRESERVE) of these cultural treasures requires significant funding and expertise. Buildings and artefacts of</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CONSIDER</t>
+          <t>preservation of these cultural treasures requires significant funding and expertise. Buildings and artefacts of (18) (CONSIDER) age must be carefully protected from the effects of time and pollution. Old city centres are particularly</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ATTRACT</t>
+          <t>considerable age must be carefully protected from the effects of time and pollution. Old city centres are particularly (19) (ATTRACT) to tourists from around the world, bringing economic benefits to local communities. Many countries invest heavily in maintaining</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TRADITION</t>
+          <t>attractive to tourists from around the world, bringing economic benefits to local communities. Many countries invest heavily in maintaining (20) (TRADITION) crafts, languages, and customs that form part of their national identity. These efforts ensure that</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>CULTURE</t>
+          <t>traditional crafts, languages, and customs that form part of their national identity. These efforts ensure that (21) (CULTURE) practices are not lost as societies modernise and change. Museums also play an important</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>EDUCATE</t>
+          <t>cultural practices are not lost as societies modernise and change. Museums also play an important (22) (EDUCATE) role, offering exhibitions that teach visitors about the past. When historic buildings are damaged, skilled craftspeople are employed to carry out sensitive</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>RESTORE</t>
+          <t>educational role, offering exhibitions that teach visitors about the past. When historic buildings are damaged, skilled craftspeople are employed to carry out sensitive (23) (RESTORE) work. The knowledge and skills passed down through generations are considered truly</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>restoration work. The knowledge and skills passed down through generations are considered truly (24) (VALUE) and irreplaceable.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1962,42 +1962,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>POISON</t>
+          <t>renewable sources of energy as a cleaner alternative to fossil fuels. Coal and oil release (17) (POISON) gases that contribute to global warming and damage air quality. Reducing our</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DEPEND</t>
+          <t>poisonous gases that contribute to global warming and damage air quality. Reducing our (18) (DEPEND) on these fuels is considered essential by most climate scientists. Solar panels and wind turbines have improved in</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EFFICIENT</t>
+          <t>dependence on these fuels is considered essential by most climate scientists. Solar panels and wind turbines have improved in (19) (EFFICIENT) over recent decades, making them far more practical. The</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ADVANCE</t>
+          <t>efficiency over recent decades, making them far more practical. The (20) (ADVANCE) of battery technology has also helped to solve the problem of storing energy when the sun is not shining. Governments are making considerable</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>INVEST</t>
+          <t>advancement of battery technology has also helped to solve the problem of storing energy when the sun is not shining. Governments are making considerable (21) (INVEST) in wind farms and solar parks to meet growing energy demands. The</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>investment in wind farms and solar parks to meet growing energy demands. The (22) (RELY) of renewable sources has improved greatly in recent years. There is now</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>reliability of renewable sources has improved greatly in recent years. There is now (23) (GLOBE) agreement that tackling climate change requires switching away from fossil fuels. Although renewable technology was once</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>EXPENSE</t>
+          <t>global agreement that tackling climate change requires switching away from fossil fuels. Although renewable technology was once (24) (EXPENSE), prices have fallen dramatically, making it accessible to many more countries.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2087,42 +2087,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>natural behaviour. The distances covered by some migrating creatures are truly (17) (FASCINATE). Monarch butterflies, for instance, travel thousands of miles to reach their</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DISTANCE</t>
+          <t>fascinating. Monarch butterflies, for instance, travel thousands of miles to reach their (18) (DISTANCE) winter habitats.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SCIENCE</t>
+          <t>distant winter habitats. (19) (SCIENCE) research has shown that animals use a variety of internal compasses, including the Earth's magnetic field, to navigate. The</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ASTONISH</t>
+          <t>scientific research has shown that animals use a variety of internal compasses, including the Earth's magnetic field, to navigate. The (20) (ASTONISH) researchers feel when studying these abilities remains as strong as ever. Animals appear to possess an extraordinary inner</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>NAVIGATE</t>
+          <t>astonishment researchers feel when studying these abilities remains as strong as ever. Animals appear to possess an extraordinary inner (21) (NAVIGATE) system that cannot yet be fully explained. Climate change and habitat loss present</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>THREAT</t>
+          <t>navigation system that cannot yet be fully explained. Climate change and habitat loss present (22) (THREAT) conditions for many migratory species. Animals that are</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ABLE</t>
+          <t>threatening conditions for many migratory species. Animals that are (23) (ABLE) to adapt to these changes may face decline or extinction. Experts warn that</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>CLIMATE</t>
+          <t>unable to adapt to these changes may face decline or extinction. Experts warn that (24) (CLIMATE) shifts could permanently disrupt migration patterns worldwide.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -2212,42 +2212,42 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PRODUCE</t>
+          <t>largely responsible for some of the most serious environmental damage caused by consumer culture. The (17) (PRODUCE) of new garments requires enormous amounts of water, energy, and raw materials. Many dyes used in manufacturing are highly</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DAMAGE</t>
+          <t>production of new garments requires enormous amounts of water, energy, and raw materials. Many dyes used in manufacturing are highly (18) (DAMAGE) to rivers and ecosystems. Western consumers have developed a culture of excessive</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CONSUME</t>
+          <t>damaging to rivers and ecosystems. Western consumers have developed a culture of excessive (19) (CONSUME), buying cheap clothes and discarding them quickly. Growing</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>consumption, buying cheap clothes and discarding them quickly. Growing (20) (AWARE) of these issues has led many shoppers to seek out ethical brands. Despite progress, some companies continue to behave in an</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>awareness of these issues has led many shoppers to seek out ethical brands. Despite progress, some companies continue to behave in an (21) (RESPONSIBLE) manner, making false claims about their environmental practices. Truly</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>ETHICS</t>
+          <t>irresponsible manner, making false claims about their environmental practices. Truly (22) (ETHICS) fashion requires transparency throughout the entire supply chain. Clothes made from natural fibres can be</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>BEAUTY</t>
+          <t>ethical fashion requires transparency throughout the entire supply chain. Clothes made from natural fibres can be (23) (BEAUTY) and long-lasting, reducing the need for frequent replacement. Experts now argue that fast fashion is simply</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>FASHION</t>
+          <t>beautiful and long-lasting, reducing the need for frequent replacement. Experts now argue that fast fashion is simply (24) (FASHION) for a society that takes environmental issues seriously.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2337,42 +2337,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WASTE</t>
+          <t>globally, one third of all food produced for human consumption is lost or thrown away each year. This (17) (WASTE) practice has serious consequences for both the planet and its people. The</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ECONOMY</t>
+          <t>wasteful practice has serious consequences for both the planet and its people. The (18) (ECONOMY) cost of discarding food runs into billions of pounds annually. Rotting food in landfill sites releases methane, a gas that is deeply</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>HARM</t>
+          <t>economic cost of discarding food runs into billions of pounds annually. Rotting food in landfill sites releases methane, a gas that is deeply (19) (HARM) to the climate. Better</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MANAGE</t>
+          <t>harmful to the climate. Better (20) (MANAGE) of food supplies, from farm to consumer, could dramatically reduce the amount wasted. The current situation is clearly</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>management of food supplies, from farm to consumer, could dramatically reduce the amount wasted. The current situation is clearly (21) (SUSTAIN), as natural resources are used to produce food that is never eaten. Part of the</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>SOLVE</t>
+          <t>unsustainable, as natural resources are used to produce food that is never eaten. Part of the (22) (SOLVE) lies in educating people about shopping and cooking more carefully. Greater</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>solution lies in educating people about shopping and cooking more carefully. Greater (23) (AWARE) of how much food households discard each week would shock most consumers. Supermarkets also need to act more</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>awareness of how much food households discard each week would shock most consumers. Supermarkets also need to act more (24) (RESPONSIBLE) by reducing promotions that encourage people to buy more than they need.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2462,42 +2462,42 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ANXIETY</t>
+          <t>increasingly being recognised as equally important as physical health. Many people experience periods of feeling (17) (ANXIETY) or low, especially during major life changes or periods of stress. Working in highly</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>STRESS</t>
+          <t>anxious or low, especially during major life changes or periods of stress. Working in highly (18) (STRESS) environments can have a serious impact on emotional wellbeing. People who are struggling should seek help from a</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>QUALIFY</t>
+          <t>stressful environments can have a serious impact on emotional wellbeing. People who are struggling should seek help from a (19) (QUALIFY) counsellor or psychologist as soon as possible. Campaigns aimed at raising public</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>qualified counsellor or psychologist as soon as possible. Campaigns aimed at raising public (20) (AWARE) have helped reduce the stigma associated with mental illness. Finding the right</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TREAT</t>
+          <t>awareness have helped reduce the stigma associated with mental illness. Finding the right (21) (TREAT) takes time, but early support usually leads to better outcomes. Many people show</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>RELUCTANT</t>
+          <t>treatment takes time, but early support usually leads to better outcomes. Many people show (22) (RELUCTANT) to ask for help, fearing the judgement of others. Building</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>CONFIDENT</t>
+          <t>reluctance to ask for help, fearing the judgement of others. Building (23) (CONFIDENT) through positive daily habits and social connections can make a real difference. With appropriate care, a full</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>RECOVER</t>
+          <t>confidence through positive daily habits and social connections can make a real difference. With appropriate care, a full (24) (RECOVER) from many mental health conditions is entirely possible.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2587,42 +2587,42 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DANGER</t>
+          <t>security of personal data has become one of the most pressing issues of the digital age. Every time we use an app or browse the internet, we leave digital traces that can reveal details about our lives. Without proper safeguards, this data can fall into (17) (DANGER) hands and be misused in various ways. Sharing personal details online always carries a</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RISK</t>
+          <t>dangerous hands and be misused in various ways. Sharing personal details online always carries a (18) (RISK) element, even when websites appear trustworthy. Companies often engage in large-scale</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>COLLECT</t>
+          <t>risky element, even when websites appear trustworthy. Companies often engage in large-scale (19) (COLLECT) of user data to improve their services or sell it to advertisers. In many countries, selling data without consent is</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LEGAL</t>
+          <t>collection of user data to improve their services or sell it to advertisers. In many countries, selling data without consent is (20) (LEGAL) and subject to heavy fines. Businesses that act in an</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>illegal and subject to heavy fines. Businesses that act in an (21) (RESPONSIBLE) way with customer information risk losing trust and facing serious legal action. Every individual has a right to</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>PRIVATE</t>
+          <t>irresponsible way with customer information risk losing trust and facing serious legal action. Every individual has a right to (22) (PRIVATE), and this right must be respected by all organisations. Stricter</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>REGULATE</t>
+          <t>privacy, and this right must be respected by all organisations. Stricter (23) (REGULATE) of data companies is needed to ensure citizens are properly protected. Governments are working to strengthen the legal</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>PROTECT</t>
+          <t>regulation of data companies is needed to ensure citizens are properly protected. Governments are working to strengthen the legal (24) (PROTECT) of individuals' digital information.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2712,42 +2712,42 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PERFORM</t>
+          <t>psychological approach to training and competition. The ability to manage nerves and stay calm under pressure can dramatically improve sporting (17) (PERFORM). Building genuine</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CONFIDENT</t>
+          <t>performance. Building genuine (18) (CONFIDENT) before a major event is just as important as physical preparation. Many champions agree that a</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>confidence before a major event is just as important as physical preparation. Many champions agree that a (19) (SUCCESS) mindset is what separates the best from the rest. Setting clear goals helps athletes measure their</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ACHIEVE</t>
+          <t>successful mindset is what separates the best from the rest. Setting clear goals helps athletes measure their (20) (ACHIEVE) and stay focused over time. Sports psychologists teach athletes to deal</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>MENTAL</t>
+          <t>achievements and stay focused over time. Sports psychologists teach athletes to deal (21) (MENTAL) with the pressure of competition, turning negative thoughts into positive ones. An athlete who is</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>mentally with the pressure of competition, turning negative thoughts into positive ones. An athlete who is (22) (FOCUS) during a competition is unlikely to perform at their best level. Maintaining</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>MOTIVATE</t>
+          <t>unfocused during a competition is unlikely to perform at their best level. Maintaining (23) (MOTIVATE) throughout a long season requires planning, rest, and strong self-belief. Intensive</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>TRAIN</t>
+          <t>motivation throughout a long season requires planning, rest, and strong self-belief. Intensive (24) (TRAIN) without psychological support can lead to burnout, leaving athletes unable to enjoy their sport.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2837,42 +2837,42 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DIVERSE</t>
+          <t>remarkable variety of life, from microscopic plankton to the largest whales on Earth. The (17) (DIVERSE) of species found in marine environments is truly extraordinary. However, many ocean creatures now face the threat of</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EXTINCT</t>
+          <t>diversity of species found in marine environments is truly extraordinary. However, many ocean creatures now face the threat of (18) (EXTINCT) due to hunting, pollution, and habitat loss. Industrial waste introduces</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>POLLUTE</t>
+          <t>extinction due to hunting, pollution, and habitat loss. Industrial waste introduces (19) (POLLUTE) into the sea that accumulate in the bodies of fish and other marine organisms. Overfishing at the current rate is clearly</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>pollutants into the sea that accumulate in the bodies of fish and other marine organisms. Overfishing at the current rate is clearly (20) (SUSTAIN), as fish populations cannot recover fast enough to meet global demand. Better</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>PROTECT</t>
+          <t>unsustainable, as fish populations cannot recover fast enough to meet global demand. Better (21) (PROTECT) of marine areas through ocean reserves has been shown to help species recover. Strong</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>GOVERN</t>
+          <t>protection of marine areas through ocean reserves has been shown to help species recover. Strong (22) (GOVERN) action is needed to enforce international laws against illegal fishing. Scientists warn that</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>government action is needed to enforce international laws against illegal fishing. Scientists warn that (23) (SIGNIFY) damage to coral reefs could make them functionally extinct within decades. Without urgent global cooperation, the future of our oceans may seem</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>HOPE</t>
+          <t>significant damage to coral reefs could make them functionally extinct within decades. Without urgent global cooperation, the future of our oceans may seem (24) (HOPE).</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2962,42 +2962,42 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BENEFIT</t>
+          <t>therapeutic effects on the mind and body. Listening to certain types of music can produce highly (17) (BENEFIT) changes in mood and emotional state. Studies confirm that music triggers strong</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EMOTION</t>
+          <t>beneficial changes in mood and emotional state. Studies confirm that music triggers strong (18) (EMOTION) responses, from joy and excitement to sadness and calm. Playing a musical instrument has also been shown to cause a</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>REDUCE</t>
+          <t>emotional responses, from joy and excitement to sadness and calm. Playing a musical instrument has also been shown to cause a (19) (REDUCE) in cortisol, the hormone linked to stress. Composers and musicians say that making music provides them with an endless source of</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>INSPIRE</t>
+          <t>reduction in cortisol, the hormone linked to stress. Composers and musicians say that making music provides them with an endless source of (20) (INSPIRE) and purpose. Research has shown that music can produce</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>inspiration and purpose. Research has shown that music can produce (21) (SIGNIFY) improvements in the memory and cognitive function of elderly patients. Many therapists now use music as a means of</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>COMMUNICATE</t>
+          <t>significant improvements in the memory and cognitive function of elderly patients. Many therapists now use music as a means of (22) (COMMUNICATE) with patients who cannot express their feelings in words. Learning to play an instrument requires practice, but the personal</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>IMPROVE</t>
+          <t>communication with patients who cannot express their feelings in words. Learning to play an instrument requires practice, but the personal (23) (IMPROVE) it brings is often remarkable. Perhaps most importantly, music creates truly</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>FORGET</t>
+          <t>improvement it brings is often remarkable. Perhaps most importantly, music creates truly (24) (FORGET) experiences that stay with people throughout their lives.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -3087,42 +3087,42 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SOPHISTICATE</t>
+          <t>criminal activities in the modern world, posing a serious threat to individuals, businesses, and governments alike. Hackers and online fraudsters are becoming increasingly (17) (SOPHISTICATE), using advanced techniques to steal data and money. Financial institutions spend billions every year on</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PROTECT</t>
+          <t>sophisticated, using advanced techniques to steal data and money. Financial institutions spend billions every year on (18) (PROTECT) against cyber attacks, yet serious breaches still occur. Accessing someone's private accounts without permission is entirely</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>LEGAL</t>
+          <t>protection against cyber attacks, yet serious breaches still occur. Accessing someone's private accounts without permission is entirely (19) (LEGAL) and can result in severe penalties. A key part of reducing cybercrime is building greater</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>illegal and can result in severe penalties. A key part of reducing cybercrime is building greater (20) (AWARE) among ordinary internet users about how to stay safe online. Acting in an</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>awareness among ordinary internet users about how to stay safe online. Acting in an (21) (RESPONSIBLE) way, such as using weak passwords or clicking unknown links, creates opportunities for criminals. Governments and technology companies are working together on strategies for the</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>PREVENT</t>
+          <t>irresponsible way, such as using weak passwords or clicking unknown links, creates opportunities for criminals. Governments and technology companies are working together on strategies for the (22) (PREVENT) of large-scale cyber attacks. The financial</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>prevention of large-scale cyber attacks. The financial (23) (SIGNIFY) damage caused by cybercrime continues to grow year on year. Building systems and networks that are fully</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>damage caused by cybercrime continues to grow year on year. Building systems and networks that are fully (24) (RELY) requires both technical expertise and constant vigilance.</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -3212,42 +3212,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HISTORY</t>
+          <t>linguistic system developed over thousands of years. The study of ancient languages provides (17) (HISTORY) insight into how early civilisations thought and organised their societies. The</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FASCINATE</t>
+          <t>historical insight into how early civilisations thought and organised their societies. The (18) (FASCINATE) with deciphering ancient scripts such as Egyptian hieroglyphics remains strong among archaeologists. Language is a deeply</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CULTURE</t>
+          <t>fascination with deciphering ancient scripts such as Egyptian hieroglyphics remains strong among archaeologists. Language is a deeply (19) (CULTURE) inheritance, carrying the stories, beliefs, and values of generations past. Tragically, many ancient languages now face</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>EXTINCT</t>
+          <t>cultural inheritance, carrying the stories, beliefs, and values of generations past. Tragically, many ancient languages now face (20) (EXTINCT) as communities abandon them in favour of global languages. Today, there are only a handful of native</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SPEAK</t>
+          <t>extinction as communities abandon them in favour of global languages. Today, there are only a handful of native (21) (SPEAK) of some of the world's rarest languages. Active efforts for the</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>PRESERVE</t>
+          <t>speakers of some of the world's rarest languages. Active efforts for the (22) (PRESERVE) of endangered languages involve recording vocabulary and creating educational materials. The loss of any language represents a</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>preservation of endangered languages involve recording vocabulary and creating educational materials. The loss of any language represents a (23) (SIGNIFY) blow to human knowledge and diversity. Without urgent action, the</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>COMMUNICATE</t>
+          <t>significant blow to human knowledge and diversity. Without urgent action, the (24) (COMMUNICATE) channels linking us to ancient civilisations may be permanently closed.</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -3337,42 +3337,42 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SCARCE</t>
+          <t>pressing global concern, as demand rises faster than natural sources can replenish. In many regions, water (17) (SCARCE) is already a daily reality that affects millions of people. Industrial and agricultural</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>POLLUTE</t>
+          <t>scarcity is already a daily reality that affects millions of people. Industrial and agricultural (18) (POLLUTE) of rivers and lakes further reduces the amount of clean water available for drinking.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>pollution of rivers and lakes further reduces the amount of clean water available for drinking. (19) (RESPONSIBLE) use of water by both individuals and industries contributes to the rapid depletion of vital reserves. In some parts of the world, the lack of access to clean water has a</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>irresponsible use of water by both individuals and industries contributes to the rapid depletion of vital reserves. In some parts of the world, the lack of access to clean water has a (20) (SIGNIFY) impact on public health and food production. The</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CONSERVE</t>
+          <t>significant impact on public health and food production. The (21) (CONSERVE) of water resources must become a global priority if future generations are to have enough clean water. Many countries now face</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>DANGER</t>
+          <t>conservation of water resources must become a global priority if future generations are to have enough clean water. Many countries now face (22) (DANGER) levels of water stress, particularly during summer droughts. Effective</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>MANAGE</t>
+          <t>dangerous levels of water stress, particularly during summer droughts. Effective (23) (MANAGE) of water infrastructure, combined with better agricultural practices, can help greatly. Moving towards a more</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>management of water infrastructure, combined with better agricultural practices, can help greatly. Moving towards a more (24) (SUSTAIN) model of water use is one of the greatest challenges facing humanity today.</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -3462,42 +3462,42 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IMAGINE</t>
+          <t>beneficial activities a person can engage in, regardless of age. Books provide a window into other worlds, firing the (17) (IMAGINE) and transporting readers to times and places they may never otherwise experience. Great literature is</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>WONDER</t>
+          <t>imagination and transporting readers to times and places they may never otherwise experience. Great literature is (18) (WONDER) in its ability to capture human emotion and experience in just a few lines. In addition to entertainment, books are an invaluable source of</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KNOW</t>
+          <t>wonderful in its ability to capture human emotion and experience in just a few lines. In addition to entertainment, books are an invaluable source of (19) (KNOW) that can inform, educate, and inspire. Reading regularly appears to satisfy an intellectual</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CURIOUS</t>
+          <t>knowledge that can inform, educate, and inspire. Reading regularly appears to satisfy an intellectual (20) (CURIOUS) that other forms of media rarely match. People who read frequently tend to show a noticeable</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>IMPROVE</t>
+          <t>curiosity that other forms of media rarely match. People who read frequently tend to show a noticeable (21) (IMPROVE) in vocabulary, writing skills, and critical thinking. For many people, reading is also a form of</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>RELAX</t>
+          <t>improvement in vocabulary, writing skills, and critical thinking. For many people, reading is also a form of (22) (RELAX) that provides a welcome escape from daily pressures. Research confirms that the</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>relaxation that provides a welcome escape from daily pressures. Research confirms that the (23) (SIGNIFY) cognitive benefits of reading continue into old age. Even in a world dominated by screens and social media, reading remains a deeply</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ENJOY</t>
+          <t>significant cognitive benefits of reading continue into old age. Even in a world dominated by screens and social media, reading remains a deeply (24) (ENJOY) and rewarding pursuit.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -3587,42 +3587,42 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DANGER</t>
+          <t>urgently needed, as thousands of species face the threat of permanent loss. Many animals, from insects to large mammals, are now considered (17) (DANGER) due to habitat destruction, hunting, and climate change. Pesticides and pollutants are deeply</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HARM</t>
+          <t>endangered due to habitat destruction, hunting, and climate change. Pesticides and pollutants are deeply (18) (HARM) to birds, insects, and aquatic life, disrupting entire ecosystems. Deforestation causes</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>harmful to birds, insects, and aquatic life, disrupting entire ecosystems. Deforestation causes (19) (SIGNIFY) damage to biodiversity hotspots where many unique species live. A more</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>significant damage to biodiversity hotspots where many unique species live. A more (20) (SUSTAIN) approach to land use and farming would allow natural habitats to recover. Charities dedicated to</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CONSERVE</t>
+          <t>sustainable approach to land use and farming would allow natural habitats to recover. Charities dedicated to (21) (CONSERVE) efforts work tirelessly to protect rare species and restore damaged environments. One of the most damaging threats to wildlife is the</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>LEGAL</t>
+          <t>conservation efforts work tirelessly to protect rare species and restore damaged environments. One of the most damaging threats to wildlife is the (22) (LEGAL) trade in animal products, which continues despite international bans. Protecting nature requires a sense of shared</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>illegal trade in animal products, which continues despite international bans. Protecting nature requires a sense of shared (23) (RESPONSIBLE) among governments, businesses, and individuals. Despite the scale of the crisis, there are still</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>HOPE</t>
+          <t>responsibility among governments, businesses, and individuals. Despite the scale of the crisis, there are still (24) (HOPE) signs, including the recovery of several previously threatened species.</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -3712,42 +3712,42 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EMPLOY</t>
+          <t>automation of many routine tasks is transforming the modern workplace. Technology is creating new areas of (17) (EMPLOY) for skilled workers, though a</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>employment for skilled workers, though a (18) (SIGNIFY) number of traditional jobs are also disappearing. Future employees will need to show</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ADAPT</t>
+          <t>significant number of traditional jobs are also disappearing. Future employees will need to show (19) (ADAPT) and qualities such as</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CREATE</t>
+          <t>adaptability and qualities such as (20) (CREATE) and critical thinking. Many companies now offer greater</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>FLEXIBLE</t>
+          <t>creativity and critical thinking. Many companies now offer greater (21) (FLEXIBLE) to attract talented staff, while individuals are increasingly seeking</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>PROFESSION</t>
+          <t>flexibility to attract talented staff, while individuals are increasingly seeking (22) (PROFESSION) development opportunities to stay relevant. Governments must also take</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>professional development opportunities to stay relevant. Governments must also take (23) (RESPONSIBLE) for retraining workers who have been affected. Investing in</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>EDUCATE</t>
+          <t>responsibility for retraining workers who have been affected. Investing in (24) (EDUCATE) is widely seen as the best way to prepare people for the changing world of work.</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3837,42 +3837,42 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>USE</t>
+          <t>growing popularity of urban farming is changing how cities think about food production. Converting (17) (USE) spaces such as rooftops and vacant lots into gardens helps improve local food</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>unused spaces such as rooftops and vacant lots into gardens helps improve local food (18) (SUSTAIN). These projects also offer</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EDUCATE</t>
+          <t>sustainability. These projects also offer (19) (EDUCATE) opportunities for residents, teaching them about nutrition and seasonal produce. Urban farms contribute to</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ENVIRONMENT</t>
+          <t>educational opportunities for residents, teaching them about nutrition and seasonal produce. Urban farms contribute to (20) (ENVIRONMENT) improvements by reducing food miles and carbon emissions. They also build a sense of</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>NEIGHBOUR</t>
+          <t>environmental improvements by reducing food miles and carbon emissions. They also build a sense of (21) (NEIGHBOUR) and help tackle food</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>SECURE</t>
+          <t>neighbourhood and help tackle food (22) (SECURE) in deprived areas. Local</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>GOVERN</t>
+          <t>insecurity in deprived areas. Local (23) (GOVERN) is increasingly supportive, offering grants to encourage this form of</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>AGRICULTURE</t>
+          <t>government is increasingly supportive, offering grants to encourage this form of (24) (AGRICULTURE) production.</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3962,42 +3962,42 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ANXIOUS</t>
+          <t>popularity of meditation has grown considerably in recent years. Many people find that regular practice reduces (17) (ANXIOUS) and helps manage the</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PRESS</t>
+          <t>anxiety and helps manage the (18) (PRESS) of daily life. Sessions can improve</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CONCENTRATE</t>
+          <t>pressures of daily life. Sessions can improve (19) (CONCENTRATE) and sharpen mental focus, making difficult tasks feel more</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>MANAGE</t>
+          <t>concentration and sharpen mental focus, making difficult tasks feel more (20) (MANAGE). Research shows that meditation promotes</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>EMOTION</t>
+          <t>manageable. Research shows that meditation promotes (21) (EMOTION) wellbeing by encouraging more</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>THOUGHT</t>
+          <t>emotional wellbeing by encouraging more (22) (THOUGHT) responses to stress. Practitioners report greater</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>PATIENT</t>
+          <t>thoughtful responses to stress. Practitioners report greater (23) (PATIENT) and a stronger sense of inner</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>RESILIENT</t>
+          <t>patience and a stronger sense of inner (24) (RESILIENT) when facing life's challenges. As a result, doctors and psychologists increasingly recommend mindfulness-based techniques to patients with a range of mental health concerns.</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -4087,42 +4087,42 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ENVIRONMENT</t>
+          <t>frequency of extreme weather events has risen sharply over recent decades. Scientists attribute this largely to human-caused (17) (ENVIRONMENT) changes, particularly the release of greenhouse gases. Rising temperatures are making storms and floods increasingly</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DESTROY</t>
+          <t>environmental changes, particularly the release of greenhouse gases. Rising temperatures are making storms and floods increasingly (18) (DESTROY). Unless governments take action to reduce carbon emissions quickly, the consequences could be</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CATASTROPHE</t>
+          <t>destructive. Unless governments take action to reduce carbon emissions quickly, the consequences could be (19) (CATASTROPHE). Communities in</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>VULNER</t>
+          <t>catastrophic. Communities in (20) (VULNER) regions will need</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CONSIDER</t>
+          <t>vulnerable regions will need (21) (CONSIDER) support to adapt. It is also important to raise</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>considerable support to adapt. It is also important to raise (22) (AWARE) among the public so that people understand the</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>awareness among the public so that people understand the (23) (URGENT) of addressing this global challenge before it is too late. Individual</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>urgency of addressing this global challenge before it is too late. Individual (24) (RESPONSIBLE) must also play a part in reducing emissions.</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -4212,42 +4212,42 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EXPENSE</t>
+          <t>invention of photography in the 19th century changed how people recorded the world around them. Early cameras were (17) (EXPENSE) and required long exposure times, but they produced images of</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EXTRA</t>
+          <t>expensive and required long exposure times, but they produced images of (18) (EXTRA) detail. Over time, technological</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>IMPROVE</t>
+          <t>extraordinary detail. Over time, technological (19) (IMPROVE) made photography more</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ACCESS</t>
+          <t>improvements made photography more (20) (ACCESS) to ordinary people. The</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>INTRODUCE</t>
+          <t>accessible to ordinary people. The (21) (INTRODUCE) of digital cameras in the late twentieth century transformed the industry once again. Today, millions of</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>PHOTOGRAPH</t>
+          <t>introduction of digital cameras in the late twentieth century transformed the industry once again. Today, millions of (22) (PHOTOGRAPH) are taken every day, often using smartphones. This has created an</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>PRECEDE</t>
+          <t>photographs are taken every day, often using smartphones. This has created an (23) (PRECEDE) visual record of human experience and sparked new debates about</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>PRIVATE</t>
+          <t>unprecedented visual record of human experience and sparked new debates about (24) (PRIVATE) and the ethics of image sharing.</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -4337,42 +4337,42 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CONFIDENT</t>
+          <t>negotiation requires a combination of skill, patience and preparation. Good negotiators demonstrate (17) (CONFIDENT) during discussions and are able to communicate their position with</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CLEAR</t>
+          <t>confidence during discussions and are able to communicate their position with (18) (CLEAR). They also show great</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>FLEXIBLE</t>
+          <t>clarity. They also show great (19) (FLEXIBLE), adapting their approach to meet the needs of all parties involved. Listening</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CAREFUL</t>
+          <t>flexibility, adapting their approach to meet the needs of all parties involved. Listening (20) (CAREFUL) is just as important as speaking, as it allows negotiators to understand what the other side truly wants. Finding</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CREATE</t>
+          <t>carefully is just as important as speaking, as it allows negotiators to understand what the other side truly wants. Finding (21) (CREATE) solutions that benefit everyone leads to more</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>DURATION</t>
+          <t>creative solutions that benefit everyone leads to more (22) (DURATION) agreements. A lack of</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>HONEST</t>
+          <t>durable agreements. A lack of (23) (HONEST) can quickly undermine trust and make it harder to reach any</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>honesty can quickly undermine trust and make it harder to reach any (24) (SATISFY) outcome for all those involved.</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -4462,42 +4462,42 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EXCITE</t>
+          <t>scientific evidence that colour can significantly affect our moods and behaviour. Researchers have found that red tends to increase (17) (EXCITE) and stimulate appetite, which is why it is commonly used in fast-food</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ADVERTISE</t>
+          <t>excitement and stimulate appetite, which is why it is commonly used in fast-food (18) (ADVERTISE). Blue, on the other hand, is often associated with feelings of</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CALM</t>
+          <t>advertising. Blue, on the other hand, is often associated with feelings of (19) (CALM) and trust. Businesses use colour</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>STRATEGY</t>
+          <t>calmness and trust. Businesses use colour (20) (STRATEGY) to influence consumer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PERCEIVE</t>
+          <t>strategically to influence consumer (21) (PERCEIVE) and encourage</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>LOYAL</t>
+          <t>perception and encourage (22) (LOYAL). Interior designers also consider colour carefully, as it can affect</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>PRODUCE</t>
+          <t>loyalty. Interior designers also consider colour carefully, as it can affect (23) (PRODUCE) in the workplace and a person's overall sense of</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>WELL</t>
+          <t>productivity in the workplace and a person's overall sense of (24) (WELL). Understanding colour psychology has become an important tool in both marketing and design.</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -4587,42 +4587,42 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>REMARK</t>
+          <t>electrification of transport is being seen as a key step in reducing carbon emissions worldwide. Sales of battery-powered cars have grown at a (17) (REMARK) rate in recent years, driven by consumer</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>remarkable rate in recent years, driven by consumer (18) (AWARE) of climate change and rising fuel costs. Governments are offering</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>FINANCE</t>
+          <t>awareness of climate change and rising fuel costs. Governments are offering (19) (FINANCE) incentives to encourage drivers to switch to cleaner vehicles. However, there are still</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>TECHNOLOGY</t>
+          <t>financial incentives to encourage drivers to switch to cleaner vehicles. However, there are still (20) (TECHNOLOGY) challenges to overcome, particularly regarding battery range and</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CHARGE</t>
+          <t>technological challenges to overcome, particularly regarding battery range and (21) (CHARGE) infrastructure. Critics also point to the</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ENVIRONMENT</t>
+          <t>charging infrastructure. Critics also point to the (22) (ENVIRONMENT) impact of mining the materials used in batteries. Despite these concerns, the overall</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>TRANSIT</t>
+          <t>environmental impact of mining the materials used in batteries. Despite these concerns, the overall (23) (TRANSIT) to electric vehicles appears</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>EVITABLE</t>
+          <t>transition to electric vehicles appears (24) (EVITABLE), as the world looks for cleaner alternatives to petrol and diesel.</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -4712,42 +4712,42 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>COGNITION</t>
+          <t>bilingualism has expanded greatly over the past few decades. Research suggests that speaking more than one language can bring significant (17) (COGNITION) benefits, such as improved memory and faster problem-solving. Children who grow up in</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MULTIPLE</t>
+          <t>cognitive benefits, such as improved memory and faster problem-solving. Children who grow up in (18) (MULTIPLE) households tend to develop stronger</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>COMMUNICATE</t>
+          <t>multilingual households tend to develop stronger (19) (COMMUNICATE) skills from an early age. Bilingualism has also been linked to</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PROFESSION</t>
+          <t>communication skills from an early age. Bilingualism has also been linked to (20) (PROFESSION) advantages in the global job market. Employers value candidates who can work across cultures with</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>SENSITIVE</t>
+          <t>professional advantages in the global job market. Employers value candidates who can work across cultures with (21) (SENSITIVE). Additionally, speaking multiple languages increases</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>CULTURE</t>
+          <t>sensitivity. Additionally, speaking multiple languages increases (22) (CULTURE) understanding and fosters greater</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>TOLERATE</t>
+          <t>cultural understanding and fosters greater (23) (TOLERATE) between people of different backgrounds. There is also growing evidence that bilingualism may reduce the risk of mental</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>DETERIORATE</t>
+          <t>tolerance between people of different backgrounds. There is also growing evidence that bilingualism may reduce the risk of mental (24) (DETERIORATE) in older adults.</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4837,42 +4837,42 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>RESPONSIBLE</t>
+          <t>global expansion of tourism has brought both opportunities and challenges for local communities. When managed (17) (RESPONSIBLE), tourism can promote cross-cultural</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>UNDERSTAND</t>
+          <t>responsibly, tourism can promote cross-cultural (18) (UNDERSTAND) and create valuable economic</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>OPPORTUNE</t>
+          <t>understanding and create valuable economic (19) (OPPORTUNE). Visitors often develop a deeper</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>APPRECIATE</t>
+          <t>opportunities. Visitors often develop a deeper (20) (APPRECIATE) for traditions and customs very different from their own. However, mass tourism can also cause</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>appreciation for traditions and customs very different from their own. However, mass tourism can also cause (21) (SIGNIFY) damage to fragile environments and local ways of life. Some communities face the</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>COMMERCE</t>
+          <t>significant damage to fragile environments and local ways of life. Some communities face the (22) (COMMERCE) of their culture, turning</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>TRADITION</t>
+          <t>commercialisation of their culture, turning (23) (TRADITION) practices into performances for tourists. To ensure</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>traditional practices into performances for tourists. To ensure (24) (SUSTAIN), governments and travel companies must work together to develop tourism models that respect and protect local heritage.</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4962,42 +4962,42 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CONNECT</t>
+          <t>complexity of human memory continues to fascinate scientists and psychologists alike. Memory is not a single process but involves multiple (17) (CONNECT) systems in the brain. Research has shown that</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>EMOTION</t>
+          <t>interconnected systems in the brain. Research has shown that (18) (EMOTION) experiences are often remembered more vividly than neutral ones, which explains why</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>emotional experiences are often remembered more vividly than neutral ones, which explains why (19) (SIGNIFY) events from childhood stay with us throughout our lives. Scientists have made</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CONSIDER</t>
+          <t>significant events from childhood stay with us throughout our lives. Scientists have made (20) (CONSIDER) progress in understanding how memories are stored and retrieved. However, memory is also</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SURPRISE</t>
+          <t>considerable progress in understanding how memories are stored and retrieved. However, memory is also (21) (SURPRISE) unreliable; it can be distorted by</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>SUGGEST</t>
+          <t>surprisingly unreliable; it can be distorted by (22) (SUGGEST) and other outside influences. Developing effective</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>STRATEGIC</t>
+          <t>suggestion and other outside influences. Developing effective (23) (STRATEGIC) for improving memory has become an important area of study, with</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>PRACTICE</t>
+          <t>strategies for improving memory has become an important area of study, with (24) (PRACTICE) applications in education, healthcare, and everyday life.</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -5087,42 +5087,42 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EXCESS</t>
+          <t>pollution is increasingly recognised as a serious public health issue in many countries. (17) (EXCESS) levels of noise from traffic, construction, and aircraft can cause stress, sleep</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>DISTURB</t>
+          <t>excessive levels of noise from traffic, construction, and aircraft can cause stress, sleep (18) (DISTURB), and even long-term hearing damage. Studies have shown that people living in noisy areas tend to be less</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>PRODUCE</t>
+          <t>disturbance, and even long-term hearing damage. Studies have shown that people living in noisy areas tend to be less (19) (PRODUCE) and more prone to anxiety. The</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PSYCHE</t>
+          <t>productive and more prone to anxiety. The (20) (PSYCHE) effects of constant noise should not be underestimated. Urban planners are now designing</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>QUIET</t>
+          <t>psychological effects of constant noise should not be underestimated. Urban planners are now designing (21) (QUIET) streets by incorporating noise barriers and green spaces.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>LEGISLATE</t>
+          <t>quieter streets by incorporating noise barriers and green spaces. (22) (LEGISLATE) requiring businesses and local authorities to reduce noise levels is also becoming more common. Raising public</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>legislation requiring businesses and local authorities to reduce noise levels is also becoming more common. Raising public (23) (AWARE) of the issue is essential so that individuals can take</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>PREVENT</t>
+          <t>awareness of the issue is essential so that individuals can take (24) (PREVENT) steps to protect their own hearing and wellbeing.</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -5212,42 +5212,42 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>REPLACE</t>
+          <t>information and learning for communities worldwide. Despite the rise of the internet, libraries remain (17) (REPLACE) spaces where people of all ages can access a wide range of resources. They provide a quiet</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ENVIRON</t>
+          <t>irreplaceable spaces where people of all ages can access a wide range of resources. They provide a quiet (18) (ENVIRON) for study and offer</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>environment for study and offer (19) (VALUE) support to those who lack internet access at home. Modern libraries also host</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>EDUCATE</t>
+          <t>valuable support to those who lack internet access at home. Modern libraries also host (20) (EDUCATE) programmes, workshops, and cultural events that bring communities together. Librarians are</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>educational programmes, workshops, and cultural events that bring communities together. Librarians are (21) (HIGH) trained professionals who help users find and evaluate</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>highly trained professionals who help users find and evaluate (22) (RELY) sources of information. Many libraries now offer digital services, demonstrating their</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>REMARK</t>
+          <t>reliable sources of information. Many libraries now offer digital services, demonstrating their (23) (REMARK) ability to adapt. Far from becoming</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>OBSOLESCENCE</t>
+          <t>remarkable ability to adapt. Far from becoming (24) (OBSOLESCENCE), libraries continue to play a vital role in promoting lifelong learning.</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -5337,42 +5337,42 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BALANCE</t>
+          <t>nutritional choices is one of the most important things a person can do for their health. A (17) (BALANCE) diet rich in fruit, vegetables, and whole grains can reduce the risk of many</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PREVENT</t>
+          <t>balanced diet rich in fruit, vegetables, and whole grains can reduce the risk of many (18) (PREVENT) diseases. However, busy modern lifestyles often make it</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>DIFFICULTY</t>
+          <t>preventable diseases. However, busy modern lifestyles often make it (19) (DIFFICULTY) for people to prepare fresh, home-cooked meals every day. The food industry also plays a</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>difficult for people to prepare fresh, home-cooked meals every day. The food industry also plays a (20) (SIGNIFY) role, as</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>HEAVY</t>
+          <t>significant role, as (21) (HEAVY) processed foods are often marketed as</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>CONVENIENCE</t>
+          <t>heavily processed foods are often marketed as (22) (CONVENIENCE) alternatives to healthy options. Public health campaigns aim to raise</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>AWARE</t>
+          <t>convenient alternatives to healthy options. Public health campaigns aim to raise (23) (AWARE) of the benefits of nutritious eating, particularly among young people. Introducing better food education in schools could make a real</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DIFFER</t>
+          <t>awareness of the benefits of nutritious eating, particularly among young people. Introducing better food education in schools could make a real (24) (DIFFER) to the nation's long-term health.</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -5462,42 +5462,42 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SOLVE</t>
+          <t>educational value of video games has grown significantly in recent years. Supporters argue that games can develop (17) (SOLVE) skills, improve</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CONCENTRATE</t>
+          <t>problem-solving skills, improve (18) (CONCENTRATE), and encourage</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CREATE</t>
+          <t>concentration, and encourage (19) (CREATE). Some studies suggest that strategic games can enhance spatial awareness and</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>DECIDE</t>
+          <t>creativity. Some studies suggest that strategic games can enhance spatial awareness and (20) (DECIDE) abilities. However, critics warn that</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>EXCESS</t>
+          <t>decision-making abilities. However, critics warn that (21) (EXCESS) screen time may have negative effects on children's</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>DEVELOP</t>
+          <t>excessive screen time may have negative effects on children's (22) (DEVELOP), particularly when it replaces physical activity or</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>PERSON</t>
+          <t>development, particularly when it replaces physical activity or (23) (PERSON) interaction. Teachers and parents must work together to ensure that gaming remains a</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>BENEFIT</t>
+          <t>interpersonal interaction. Teachers and parents must work together to ensure that gaming remains a (24) (BENEFIT) and controlled part of a child's education rather than a harmful distraction.</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -5587,42 +5587,42 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>expansion of e-commerce over the past two decades has transformed the way people shop. Online (17) (RETAIL) now offer a vast range of products at</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COMPETE</t>
+          <t>retailers now offer a vast range of products at (18) (COMPETE) prices, making it easy for consumers to compare options and find what they need. The</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>CONVENIENT</t>
+          <t>competitive prices, making it easy for consumers to compare options and find what they need. The (19) (CONVENIENT) of shopping from home has led millions of people to abandon traditional high streets. Despite its many</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ADVANTAGE</t>
+          <t>convenience of shopping from home has led millions of people to abandon traditional high streets. Despite its many (20) (ADVANTAGE), e-commerce has also raised concerns about</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>EMPLOY</t>
+          <t>advantages, e-commerce has also raised concerns about (21) (EMPLOY) in the retail sector, as many physical stores have closed. There are also growing worries about</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>ENVIRONMENT</t>
+          <t>employment in the retail sector, as many physical stores have closed. There are also growing worries about (22) (ENVIRONMENT) impacts, since increased delivery traffic contributes to carbon emissions. Companies are now under</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>CONSIDER</t>
+          <t>environmental impacts, since increased delivery traffic contributes to carbon emissions. Companies are now under (23) (CONSIDER) pressure to find more</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>SUSTAIN</t>
+          <t>considerable pressure to find more (24) (SUSTAIN) solutions, such as electric delivery vehicles and reduced packaging.</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -5712,42 +5712,42 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ENVIRONMENT</t>
+          <t>sustainability is now central to modern architectural design and urban planning. Architects are increasingly focused on creating buildings that are (17) (ENVIRONMENT) friendly and energy-efficient. The use of</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>RENEW</t>
+          <t>environmentally friendly and energy-efficient. The use of (18) (RENEW) materials such as timber and bamboo is becoming more common, as is the</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>INSTALL</t>
+          <t>renewable materials such as timber and bamboo is becoming more common, as is the (19) (INSTALL) of solar panels and green roofs. Such</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>INNOVATE</t>
+          <t>installation of solar panels and green roofs. Such (20) (INNOVATE) designs can significantly reduce a building's carbon footprint. They can also improve the</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>WELL</t>
+          <t>innovative designs can significantly reduce a building's carbon footprint. They can also improve the (21) (WELL) of occupants by providing natural light and better air quality. Critics argue that sustainable building methods can be</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>EXPENSE</t>
+          <t>wellbeing of occupants by providing natural light and better air quality. Critics argue that sustainable building methods can be (22) (EXPENSE), though costs are falling as technologies improve. In the long term, the</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>ECONOMY</t>
+          <t>expensive, though costs are falling as technologies improve. In the long term, the (23) (ECONOMY) benefits of energy-efficient buildings are clear, making sustainability a</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>WORTH</t>
+          <t>economic benefits of energy-efficient buildings are clear, making sustainability a (24) (WORTH) investment for property owners and society alike.</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -5837,42 +5837,42 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SIGNIFY</t>
+          <t>physically active is vital for both body and mind. Studies show that regular outdoor exercise leads to (17) (SIGNIFY) improvements in cardiovascular health and overall</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>FIT</t>
+          <t>significant improvements in cardiovascular health and overall (18) (FIT). Activities such as hiking, cycling, and swimming build</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ENDURE</t>
+          <t>fitness. Activities such as hiking, cycling, and swimming build (19) (ENDURE) and strengthen muscles, while also helping people to maintain a</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>HEALTH</t>
+          <t>endurance and strengthen muscles, while also helping people to maintain a (20) (HEALTH) weight. Beyond the physical benefits, spending time in nature has a</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>healthy weight. Beyond the physical benefits, spending time in nature has a (21) (POWER) effect on mental health. Exposure to green spaces has been linked to reduced stress levels and improved</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>CONCENTRATE</t>
+          <t>powerful effect on mental health. Exposure to green spaces has been linked to reduced stress levels and improved (22) (CONCENTRATE). Despite this, many people lead increasingly</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>SEDATE</t>
+          <t>concentration. Despite this, many people lead increasingly (23) (SEDATE) lives and fail to get the amount of</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>DAY</t>
+          <t>sedentary lives and fail to get the amount of (24) (DAY) exercise recommended by health professionals, often citing a lack of time or motivation.</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -5962,42 +5962,42 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CONGEST</t>
+          <t>efficiency of public transport systems is one of the most effective ways to reduce urban congestion. Well-designed networks can significantly reduce (17) (CONGEST) and cut both air</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>POLLUTE</t>
+          <t>congestion and cut both air (18) (POLLUTE) and carbon emissions. Passengers also benefit from lower</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>pollution and carbon emissions. Passengers also benefit from lower (19) (TRANSPORT) costs compared to owning and running a private car. However, many cities still struggle with</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>transportation costs compared to owning and running a private car. However, many cities still struggle with (20) (RELY) services and</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>SUFFICIENT</t>
+          <t>unreliable services and (21) (SUFFICIENT) funding to maintain ageing</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>STRUCTURE</t>
+          <t>insufficient funding to maintain ageing (22) (STRUCTURE). Governments must make</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>SUBSTANCE</t>
+          <t>infrastructure. Governments must make (23) (SUBSTANCE) investment in public transport if they wish to create truly sustainable cities.</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>COURAGE</t>
+          <t>substantial investment in public transport if they wish to create truly sustainable cities. (24) (COURAGE) more people to leave their cars at home could make a real difference to urban air quality and quality of life.</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -6087,42 +6087,42 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>VARY</t>
+          <t>scientific understanding of nutrition has advanced enormously in recent decades. We now know that a (17) (VARY) diet containing plenty of fresh produce is essential for maintaining good health. Nutritionists recommend limiting the</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CONSUME</t>
+          <t>varied diet containing plenty of fresh produce is essential for maintaining good health. Nutritionists recommend limiting the (18) (CONSUME) of ultra-processed foods, which are often high in sugar, salt, and</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>HEALTH</t>
+          <t>consumption of ultra-processed foods, which are often high in sugar, salt, and (19) (HEALTH) fats. Research has revealed that the gut microbiome plays a crucial role in overall health and</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>IMMUNE</t>
+          <t>unhealthy fats. Research has revealed that the gut microbiome plays a crucial role in overall health and (20) (IMMUNE). What we eat directly affects our mood, energy levels, and</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>COGNITION</t>
+          <t>immunity. What we eat directly affects our mood, energy levels, and (21) (COGNITION) function. Despite this</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>GROW</t>
+          <t>cognitive function. Despite this (22) (GROW) body of evidence, many people find it</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>DIFFICULTY</t>
+          <t>growing body of evidence, many people find it (23) (DIFFICULTY) to change their eating habits due to busy lifestyles, food marketing, and limited access to</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>AFFORD</t>
+          <t>difficult to change their eating habits due to busy lifestyles, food marketing, and limited access to (24) (AFFORD) fresh produce.</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -6212,42 +6212,42 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CULTURE</t>
+          <t>diversity in the workplace has become a priority for many organisations around the world. Teams made up of people from different (17) (CULTURE) backgrounds bring a wider range of perspectives and ideas. This can lead to greater</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CREATE</t>
+          <t>cultural backgrounds bring a wider range of perspectives and ideas. This can lead to greater (18) (CREATE) and more effective problem-solving. Research shows that</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>creativity and more effective problem-solving. Research shows that (19) (INCLUDE) companies tend to be more</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>INNOVATE</t>
+          <t>inclusive companies tend to be more (20) (INNOVATE) and better able to serve customers from a range of backgrounds. However, creating a truly</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>WELCOME</t>
+          <t>innovative and better able to serve customers from a range of backgrounds. However, creating a truly (21) (WELCOME) workplace takes effort. Employers must address</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>EQUAL</t>
+          <t>welcoming workplace takes effort. Employers must address (22) (EQUAL) in hiring and promotion, and provide</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TRAIN</t>
+          <t>inequality in hiring and promotion, and provide (23) (TRAIN) to help staff understand and appreciate different cultural norms. When done</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>EFFECT</t>
+          <t>training to help staff understand and appreciate different cultural norms. When done (24) (EFFECT), diversity initiatives benefit not just individuals but the organisation as a whole.</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -6337,42 +6337,42 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PSYCHOLOGY</t>
+          <t>advertising industry spends billions of pounds each year trying to influence what we buy. Marketers use (17) (PSYCHOLOGY) techniques to persuade consumers to choose one product over another. Eye-catching</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>IMAGE</t>
+          <t>psychological techniques to persuade consumers to choose one product over another. Eye-catching (18) (IMAGE) and catchy slogans are</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>DELIBERATE</t>
+          <t>imagery and catchy slogans are (19) (DELIBERATE) designed to create positive</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ASSOCIATE</t>
+          <t>deliberately designed to create positive (20) (ASSOCIATE) with a brand. Critics argue that some advertising is</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>MISLEAD</t>
+          <t>associations with a brand. Critics argue that some advertising is (21) (MISLEAD), particularly when it targets children who lack the</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>CRITIC</t>
+          <t>misleading, particularly when it targets children who lack the (22) (CRITIC) skills to evaluate what they see. There are growing calls for tighter</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>REGULATE</t>
+          <t>critical skills to evaluate what they see. There are growing calls for tighter (23) (REGULATE) of advertising, especially on social media platforms. Others counter that advertising plays an important</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>ECONOMY</t>
+          <t>regulation of advertising, especially on social media platforms. Others counter that advertising plays an important (24) (ECONOMY) role by funding free media content and helping businesses grow.</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -6462,42 +6462,42 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>REASON</t>
+          <t>homelessness remains a persistent and deeply troubling problem. People become homeless for a wide variety of (17) (REASON), including</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>EMPLOY</t>
+          <t>reasons, including (18) (EMPLOY), relationship breakdown, and mental health difficulties. The consequences of sleeping rough are</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>DEVASTATE</t>
+          <t>unemployment, relationship breakdown, and mental health difficulties. The consequences of sleeping rough are (19) (DEVASTATE), affecting both physical and mental health, and making it</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>EXTREME</t>
+          <t>devastating, affecting both physical and mental health, and making it (20) (EXTREME) difficult to escape the cycle. Charities and</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>VOLUNTEER</t>
+          <t>extremely difficult to escape the cycle. Charities and (21) (VOLUNTEER) organisations provide vital support, but long-term solutions require greater</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>GOVERN</t>
+          <t>voluntary organisations provide vital support, but long-term solutions require greater (22) (GOVERN) involvement. Building more</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>AFFORD</t>
+          <t>government involvement. Building more (23) (AFFORD) housing and improving access to mental health services are two key priorities. Tackling homelessness requires a</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>COORDINATE</t>
+          <t>affordable housing and improving access to mental health services are two key priorities. Tackling homelessness requires a (24) (COORDINATE) effort from housing authorities, health services, and employers working closely together.</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -6587,42 +6587,42 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ENVIRONMENT</t>
+          <t>communal gardens are springing up in cities around the world, transforming unused land into vibrant green spaces. These projects offer a wide range of (17) (ENVIRONMENT) benefits, such as improving air quality and reducing the urban heat island effect. Growing fruit and vegetables</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>environmental benefits, such as improving air quality and reducing the urban heat island effect. Growing fruit and vegetables (18) (LOCAL) also reduces the need to transport food long distances, lowering carbon emissions. Community gardens are equally</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>locally also reduces the need to transport food long distances, lowering carbon emissions. Community gardens are equally (19) (VALUE) for social wellbeing. They bring together people of all ages, creating a sense of</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>BELONG</t>
+          <t>valuable for social wellbeing. They bring together people of all ages, creating a sense of (20) (BELONG) and shared purpose. Participants report that regular gardening can be deeply</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>THERAPY</t>
+          <t>belonging and shared purpose. Participants report that regular gardening can be deeply (21) (THERAPY) and helps to combat feelings of</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>LONELY</t>
+          <t>therapeutic and helps to combat feelings of (22) (LONELY). Working alongside others also promotes a spirit of</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>COOPERATE</t>
+          <t>loneliness. Working alongside others also promotes a spirit of (23) (COOPERATE) and improves</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>PERSON</t>
+          <t>cooperation and improves (24) (PERSON) relationships.</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -6712,42 +6712,42 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>KNOW</t>
+          <t>technological change is reshaping education systems around the world. Online learning platforms and digital tools are making (17) (KNOW) more accessible than ever before, allowing students to study at their own pace regardless of location.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>INTERACT</t>
+          <t>knowledge more accessible than ever before, allowing students to study at their own pace regardless of location. (18) (INTERACT) software can adapt to the needs of individual learners, providing a more</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>PERSONAL</t>
+          <t>interactive software can adapt to the needs of individual learners, providing a more (19) (PERSONAL) experience than traditional classroom teaching. However, the</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>WIDE</t>
+          <t>personalised experience than traditional classroom teaching. However, the (20) (WIDE) adoption of technology in education also raises concerns. Many teachers argue that face-to-face</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>INTERACT</t>
+          <t>widespread adoption of technology in education also raises concerns. Many teachers argue that face-to-face (21) (INTERACT) is essential for developing social skills and emotional intelligence. There are also worries about the</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>INCREASE</t>
+          <t>interaction is essential for developing social skills and emotional intelligence. There are also worries about the (22) (INCREASE) amount of time students spend on screens. Experts agree that the most</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>EFFECT</t>
+          <t>increasing amount of time students spend on screens. Experts agree that the most (23) (EFFECT) approach is to combine digital tools with</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>TRADITION</t>
+          <t>effective approach is to combine digital tools with (24) (TRADITION) teaching methods, creating a balanced and stimulating learning environment.</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">

</xml_diff>